<commit_message>
real villain wiz, saucer light changes
</commit_message>
<xml_diff>
--- a/docs/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
+++ b/docs/ASM67_55_Villains_11_Wizards_1_Final_Wizard_Tracker.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R34a77ac285234863"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Rc16bc61e7de74796"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Re5092d2320bc46bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="Rc06c67e2d1664cfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="R9eed8e0752954f47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="Rf12cd729add743c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R34d40fef6b934050"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rddec6cfd2af04354"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R1d7c1db78c4a458d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R65c43f2ac8854af9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="R39b78bf26e4d4109"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="Rda63c53c48674cf1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R5d379c58fd4b45a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R707fb3d418b94d29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Plan" sheetId="2" r:id="Rc5954cdef6b347b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mini-Wizards" sheetId="3" r:id="Rbc8a5fc8ab014553"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repurposed Modes" sheetId="4" r:id="Racd8d315d20d4d69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Rules Snapshot" sheetId="5" r:id="Reb10640b40fd49eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Case Files" sheetId="6" r:id="R936babb558b74276"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Todos" sheetId="7" r:id="R0bac06c09d1e4fd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rfd298c58804346c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chapter Bonuses" sheetId="9" r:id="R1f08e155857145d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Balance" sheetId="10" r:id="R49b3288178514f4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Var Cleanup" sheetId="11" r:id="Rff34cd7603c34ad6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Status" sheetId="12" r:id="R85d6a3c043f34174"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Music Inventory" sheetId="13" r:id="R1efac7caba3e45c1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4932,10 +4932,8 @@
           <x:t xml:space="preserve">Mad Science Meltdown</x:t>
         </x:is>
       </x:c>
-      <x:c r="E8" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Placeholder shell — full design/coding required</x:t>
-        </x:is>
+      <x:c r="E8" s="31" t="str">
+        <x:v>Approved/coded — needs machine playtest/polish</x:v>
       </x:c>
       <x:c r="F8" s="85" t="n"/>
       <x:c r="G8" s="85" t="n"/>
@@ -5060,10 +5058,8 @@
           <x:t xml:space="preserve">Who Is the Real Villain?</x:t>
         </x:is>
       </x:c>
-      <x:c r="E11" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Placeholder shell — full design/coding required</x:t>
-        </x:is>
+      <x:c r="E11" s="31" t="str">
+        <x:v>Implemented — needs machine playtest/polish</x:v>
       </x:c>
       <x:c r="F11" s="85" t="n"/>
       <x:c r="G11" s="85" t="n"/>
@@ -10201,10 +10197,8 @@
           <x:t xml:space="preserve">No individual Case File powers. Each Jackpot and Super Jackpot adds 20K × the chapter's collected Case Files (0–25 files; 0–500K). Ordinary switch, spinner, target, progress, and other non-jackpot scoring do not receive this bonus.</x:t>
         </x:is>
       </x:c>
-      <x:c r="G11" s="31" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Explicit placeholder shell; full design and coding required.</x:t>
-        </x:is>
+      <x:c r="G11" s="31" t="str">
+        <x:v>Implemented repeating 2-ball investigation multiball: hit both pops to reveal one random no-repeat Cameo pair (A/B, slings, or bank rubbers); rubber pair is exposed one bank drop per upper-spinner spin. Any flashing saucer reveals the correct Cameo target; early candidate hits score 100K with Daily Bugle impostor audio; correct Cameo scores 1M + Case Files. Desperado requires all five unique right drops at 50K with bank reset after every hit and upper-spinner spotting. Brutus lights all three saucers; left-bank hit closes them, right-bank hit relights them; any lit saucer scores 500K + Case Files. Then gate opens for a 20s 2M + Case Files VUK Super; collect or miss returns to Cameo. Global upper L/C/R completion adds a ball to a four-ball max with 15s save, or 500K + Case Files at cap. Needs machine playtest/polish.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -13774,12 +13768,10 @@
         </x:is>
       </x:c>
       <x:c r="C14" s="45" t="str">
-        <x:v>Review 3 functional/provisional mini-wizards; fully design and code 5 remaining placeholder shells; complete the dedicated Kingpin Final Showdown design/retheme. The Web Tightens is approved/coded and needs machine playtest. Wizard Case Files add 20K each to qualifying Jackpot values (max +500K per 1X JP).</x:v>
-      </x:c>
-      <x:c r="D14" s="45" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Future</x:t>
-        </x:is>
+        <x:v>Review remaining functional/provisional mini-wizards; fully design and code the 1 remaining placeholder shell (Time-Tossed Showdown); complete the dedicated Kingpin Final Showdown design/retheme. Who Is the Real Villain? is implemented and needs machine playtest. Wizard Case Files add 20K each to qualifying Jackpot values (max +500K per 1X JP).</x:v>
+      </x:c>
+      <x:c r="D14" s="45" t="str">
+        <x:v>In progress</x:v>
       </x:c>
     </x:row>
     <x:row r="15" s="26" customFormat="1" ht="38" customHeight="1">

</xml_diff>